<commit_message>
Add jsw-blogs, jsw-tech-showcase, parallax-collage blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 10
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-jsw-phase-3.report.xlsx
+++ b/tools/importer/reports/import-jsw-phase-3.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="36">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>cards</t>
+  </si>
+  <si>
+    <t>images</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -76,16 +82,34 @@
     <t>MG Latest Luxury &amp; Electric Cars in India - Prices &amp; Models</t>
   </si>
   <si>
+    <t>jsw-nev-collage.report.json</t>
+  </si>
+  <si>
+    <t>jsw-nev-collage</t>
+  </si>
+  <si>
+    <t>2026-10-09T10:52:29.321Z</t>
+  </si>
+  <si>
+    <t>https://example.com/</t>
+  </si>
+  <si>
     <t>jsw-phase-3.report.json</t>
   </si>
   <si>
     <t>jsw-phase-3</t>
   </si>
   <si>
-    <t>2026-10-08T18:29:38.918Z</t>
-  </si>
-  <si>
-    <t>https://example.com/</t>
+    <t>2026-10-12T08:33:57.614Z</t>
+  </si>
+  <si>
+    <t>jsw-sustainability.report.json</t>
+  </si>
+  <si>
+    <t>jsw-sustainability</t>
+  </si>
+  <si>
+    <t>2026-10-09T04:31:36.798Z</t>
   </si>
   <si>
     <t>nav.report.json</t>
@@ -483,20 +507,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="3" max="3" width="7" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="29" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="10" width="50" customWidth="1"/>
+    <col min="11" max="11" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -524,125 +550,225 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2">
         <v>4</v>
       </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
       </c>
       <c r="H3" t="s">
         <v>20</v>
       </c>
       <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
         <v>14</v>
       </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" t="s">
-        <v>24</v>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" t="s">
         <v>26</v>
       </c>
-      <c r="D5">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7">
         <v>5</v>
       </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" t="s">
+      <c r="G7" t="s">
         <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>